<commit_message>
Update regression baselines for canonical release IDs
</commit_message>
<xml_diff>
--- a/tests/regression/baseline/Traceability_Reconciliation_2026.04.xlsx
+++ b/tests/regression/baseline/Traceability_Reconciliation_2026.04.xlsx
@@ -501,7 +501,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -545,7 +545,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -589,7 +589,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -633,7 +633,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -773,7 +773,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -821,7 +821,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -955,7 +955,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1005,7 +1005,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1055,7 +1055,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1105,7 +1105,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1275,7 +1275,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1333,7 +1333,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1469,16 +1469,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
@@ -1487,10 +1492,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>RLSE1000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>STRY1000001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>EX01</t>
         </is>
@@ -1499,10 +1509,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>RLSE1000001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>STRY1000001</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>EX02</t>
         </is>
@@ -1511,10 +1526,15 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>RLSE1000001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>STRY1000001</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>EX03</t>
         </is>
@@ -1523,10 +1543,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>RLSE1000001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>STRY1000002</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>EX10</t>
         </is>
@@ -1535,10 +1560,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>RLSE1000001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>STRY1000002</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>EX11</t>
         </is>
@@ -1547,10 +1577,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>RLSE1000001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>STRY1000002</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>EX12</t>
         </is>
@@ -1559,10 +1594,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>RLSE1000001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>STRY1000003</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>EX20</t>
         </is>
@@ -1571,10 +1611,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>RLSE1000001</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>STRY1000003</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>EX21</t>
         </is>
@@ -1583,10 +1628,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>STRY2000001</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>AU01</t>
         </is>
@@ -1595,10 +1645,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>STRY2000001</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>AU02</t>
         </is>
@@ -1607,10 +1662,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>STRY2000001</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>AU03</t>
         </is>
@@ -1619,10 +1679,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>STRY2000001</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>AU04</t>
         </is>
@@ -1631,10 +1696,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>STRY2000001</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>AU05</t>
         </is>
@@ -1643,10 +1713,15 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>STRY2000002</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>AU10</t>
         </is>
@@ -1655,10 +1730,15 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>STRY2000002</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>AU11</t>
         </is>
@@ -1667,10 +1747,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>STRY2000002</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>AU12</t>
         </is>
@@ -1679,10 +1764,15 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>STRY2000003</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>AU20</t>
         </is>
@@ -1691,10 +1781,15 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>STRY2000003</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>AU21</t>
         </is>
@@ -1703,10 +1798,15 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>STRY2000004</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>AU30</t>
         </is>
@@ -1715,10 +1815,15 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>STRY2000004</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>AU31</t>
         </is>
@@ -1727,10 +1832,15 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>STRY2000005</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>AU40</t>
         </is>
@@ -1739,10 +1849,15 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>STRY2000005</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>AU41</t>
         </is>
@@ -1751,10 +1866,15 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>STRY2000005</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>AU42</t>
         </is>
@@ -2835,7 +2955,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2877,7 +2997,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2919,7 +3039,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2961,7 +3081,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3003,7 +3123,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3045,7 +3165,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3087,7 +3207,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3129,7 +3249,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RLSE1000001 Extraction Validation</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3171,7 +3291,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3213,7 +3333,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3255,7 +3375,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3297,7 +3417,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3339,7 +3459,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3381,7 +3501,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3423,7 +3543,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3465,7 +3585,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3507,7 +3627,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3549,7 +3669,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3591,7 +3711,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3633,7 +3753,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3675,7 +3795,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3705,7 +3825,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3747,7 +3867,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3789,7 +3909,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RLSE1000002 Audit Validation</t>
+          <t>RLSE1000002</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3860,7 +3980,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EX01, EX02, EX03</t>
+          <t>STRY1000001 Basic extraction of single tests EX01, EX02, EX03</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3997,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>EX10, EX11, EX12</t>
+          <t>STRY1000002 Multi-sheet extraction EX10, EX11, EX12</t>
         </is>
       </c>
     </row>
@@ -3894,7 +4014,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>EX20, EX21</t>
+          <t>STRY1000003 Cross-sheet reuse EX20, EX21</t>
         </is>
       </c>
     </row>
@@ -3911,7 +4031,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AU01 – AU05</t>
+          <t>STRY2000001 Range expansion validation AU01 – AU05</t>
         </is>
       </c>
     </row>
@@ -3928,7 +4048,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AU10, AU11, AU12</t>
+          <t>STRY2000002 Missing tests scenario AU10, AU11, AU12</t>
         </is>
       </c>
     </row>
@@ -3945,7 +4065,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AU20, AU21</t>
+          <t>STRY2000003 Misalignment scenario AU20, AU21</t>
         </is>
       </c>
     </row>
@@ -3962,7 +4082,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AU30, AU31</t>
+          <t>STRY2000004 Duplicate / cross-story tests AU30, AU31</t>
         </is>
       </c>
     </row>
@@ -3979,7 +4099,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AU40, AU41, AU42</t>
+          <t>STRY2000005 Execution Status Handling AU40, AU41, AU42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand regression spreadsheet to include new test cases
</commit_message>
<xml_diff>
--- a/tests/regression/baseline/Traceability_Reconciliation_2026.04.xlsx
+++ b/tests/regression/baseline/Traceability_Reconciliation_2026.04.xlsx
@@ -21,16 +21,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$L$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Traceability_Matrix'!$A$1:$K$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Traceability Gaps'!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$L$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Traceability_Matrix'!$A$1:$K$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Traceability Gaps'!$A$1:$N$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Missing'!$A$1:$A$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Extra'!$A$1:$A$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Extra'!$A$1:$A$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Story_To_Test_Map'!$A$1:$C$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Execution_Attachments'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Execution_Attachments'!$A$1:$H$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Execution_Detail'!$A$1:$H$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plan_Raw'!$A$1:$C$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Exec_Raw'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Exec_Raw'!$A$1:$H$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -801,13 +801,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -1979,20 +1979,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Phase A</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>STRY1000001</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>EX01</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2002,17 +2002,17 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Evidenced</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>EX02</t>
+          <t>EX01</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>EX03</t>
+          <t>EX02</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2099,20 +2099,20 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Phase B</t>
+          <t>Phase A</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>STRY1000002</t>
+          <t>STRY1000001</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>EX10</t>
+          <t>EX03</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>EX11</t>
+          <t>EX10</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>EX12</t>
+          <t>EX11</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2223,16 +2223,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>STRY1000003</t>
+          <t>STRY1000002</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>EX20</t>
+          <t>EX12</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2263,41 +2263,81 @@
         </is>
       </c>
       <c r="B37" t="n">
+        <v>5</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>STRY1000003</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>EX20</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Evidenced</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Phase B</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
         <v>6</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>STRY1000003</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>EX21</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
         <is>
           <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>Evidenced</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H37"/>
+  <autoFilter ref="A1:H38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2308,13 +2348,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
     <col width="72" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -2987,8 +3027,56 @@
         <v>0</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>STRY3999999</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>🔴 Story missing from spec</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>🔴 Passed but missing evidence</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Execution-only story: TP-ORPHAN-01</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L14"/>
+  <autoFilter ref="A1:L15"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
@@ -3015,6 +3103,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3026,12 +3115,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -3273,22 +3362,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dynamic Scheduling and Schedule Optimisation</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>STRY3000002</t>
-        </is>
-      </c>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>IS70A</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>STRY3000002</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3303,17 +3388,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>EXECUTION_ONLY</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -3340,7 +3425,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>IS70B</t>
+          <t>IS70A</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3397,7 +3482,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>IS70C</t>
+          <t>IS70B</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3454,7 +3539,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>IS70D</t>
+          <t>IS70C</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3506,17 +3591,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>STRY3000003</t>
+          <t>STRY3000002</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TP-OPT-01</t>
+          <t>IS70D</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>STRY3000003</t>
+          <t>STRY3000002</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3558,22 +3643,18 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dynamic Scheduling and Schedule Optimisation</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>STRY3000003</t>
-        </is>
-      </c>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>TP-OPT-01</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>STRY3000005</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3588,7 +3669,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -3598,7 +3679,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>MISALIGNED</t>
+          <t>EXECUTION_ONLY</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -3625,7 +3706,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TP-OPT-02</t>
+          <t>TP-OPT-01</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -3682,12 +3763,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>TP-OPT-03</t>
+          <t>TP-OPT-01</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>STRY3000003</t>
+          <t>STRY3000005</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3707,12 +3788,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>MISALIGNED</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -3734,58 +3815,74 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>STRY3000004</t>
+          <t>STRY3000003</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TP-MISS-01</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>TP-OPT-02</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>STRY3000003</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>NOT EXECUTED</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>NOT_EXECUTED</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>NOT_EXECUTED</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>DS and Optimisation</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RLSE1000001</t>
+          <t>Dynamic Scheduling and Schedule Optimisation</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>STRY1000001</t>
+          <t>STRY3000003</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>EX01</t>
+          <t>TP-OPT-03</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>STRY1000001</t>
+          <t>STRY3000003</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -3815,34 +3912,30 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Phase A</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RLSE1000001</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>STRY1000001</t>
-        </is>
-      </c>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>EX02</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>STRY1000001</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3857,106 +3950,86 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>EXECUTION_ONLY</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Phase A</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RLSE1000001</t>
+          <t>Dynamic Scheduling and Schedule Optimisation</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>STRY1000001</t>
+          <t>STRY3000004</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>EX03</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>STRY1000001</t>
-        </is>
-      </c>
+          <t>TP-MISS-01</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>NOT EXECUTED</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>NOT_EXECUTED</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Phase A</t>
-        </is>
-      </c>
+          <t>NOT_EXECUTED</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RLSE1000001</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>STRY1000002</t>
-        </is>
-      </c>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EX10</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>STRY1000002</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3971,49 +4044,45 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>EXECUTION_ONLY</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Phase B</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RLSE1000001</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>STRY1000002</t>
-        </is>
-      </c>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EX11</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>STRY1000002</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -4028,27 +4097,27 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>EXECUTION_ONLY</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Phase B</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
     </row>
@@ -4060,17 +4129,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>STRY1000002</t>
+          <t>STRY1000001</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>EX12</t>
+          <t>EX01</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>STRY1000002</t>
+          <t>STRY1000001</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -4105,7 +4174,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Phase B</t>
+          <t>Phase A</t>
         </is>
       </c>
     </row>
@@ -4117,17 +4186,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>STRY1000003</t>
+          <t>STRY1000001</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EX20</t>
+          <t>EX02</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>STRY1000003</t>
+          <t>STRY1000001</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -4162,7 +4231,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Phase B</t>
+          <t>Phase A</t>
         </is>
       </c>
     </row>
@@ -4174,17 +4243,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>STRY1000003</t>
+          <t>STRY1000001</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EX21</t>
+          <t>EX03</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>STRY1000003</t>
+          <t>STRY1000001</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -4219,29 +4288,25 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Phase B</t>
+          <t>Phase A</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RLSE1000002</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>STRY2000001</t>
-        </is>
-      </c>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AU01</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>STRY2000001</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4256,49 +4321,49 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>EXECUTION_ONLY</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Revised Core</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RLSE1000002</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>STRY2000001</t>
+          <t>STRY1000002</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AU02</t>
+          <t>EX10</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>STRY2000001</t>
+          <t>STRY1000002</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -4328,34 +4393,34 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Revised Core</t>
+          <t>Phase B</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RLSE1000002</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>STRY2000001</t>
+          <t>STRY1000002</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AU03</t>
+          <t>EX11</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>STRY2000001</t>
+          <t>STRY1000002</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -4385,34 +4450,34 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Revised Core</t>
+          <t>Phase B</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RLSE1000002</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>STRY2000001</t>
+          <t>STRY1000002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AU04</t>
+          <t>EX12</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>STRY2000001</t>
+          <t>STRY1000002</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -4442,39 +4507,35 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Revised Core</t>
+          <t>Phase B</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RLSE1000002</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>STRY2000001</t>
-        </is>
-      </c>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AU05</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>STRY2000001</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -4484,49 +4545,49 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>EXECUTION_ONLY</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Revised Core</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RLSE1000002</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>STRY2000002</t>
+          <t>STRY1000003</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AU10</t>
+          <t>EX20</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>STRY2000002</t>
+          <t>STRY1000003</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -4556,34 +4617,34 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Revised Edge Cases</t>
+          <t>Phase B</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RLSE1000002</t>
+          <t>RLSE1000001</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>STRY2000002</t>
+          <t>STRY1000003</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AU11</t>
+          <t>EX21</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>STRY2000002</t>
+          <t>STRY1000003</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -4613,34 +4674,30 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Revised Edge Cases</t>
+          <t>Phase B</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RLSE1000002</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>STRY2000002</t>
-        </is>
-      </c>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AU12</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NEGATIVE</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -4655,7 +4712,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -4665,17 +4722,17 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>MISALIGNED</t>
+          <t>EXECUTION_ONLY</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Revised Edge Cases</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
     </row>
@@ -4687,17 +4744,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>STRY2000003</t>
+          <t>STRY2000001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AU20</t>
+          <t>AU01</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>STRY2000003</t>
+          <t>STRY2000001</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -4732,7 +4789,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Revised Edge Cases</t>
+          <t>Revised Core</t>
         </is>
       </c>
     </row>
@@ -4744,17 +4801,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>STRY2000003</t>
+          <t>STRY2000001</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AU21</t>
+          <t>AU02</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>STRY2000004</t>
+          <t>STRY2000001</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -4774,12 +4831,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>MISALIGNED</t>
+          <t>ALIGNED</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -4789,7 +4846,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Revised Edge Cases</t>
+          <t>Revised Core</t>
         </is>
       </c>
     </row>
@@ -4801,17 +4858,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>STRY2000004</t>
+          <t>STRY2000001</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AU30</t>
+          <t>AU03</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>STRY2000004</t>
+          <t>STRY2000001</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -4846,7 +4903,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Revised Edge Cases</t>
+          <t>Revised Core</t>
         </is>
       </c>
     </row>
@@ -4858,17 +4915,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>STRY2000004</t>
+          <t>STRY2000001</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AU30</t>
+          <t>AU04</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>STRY2000002</t>
+          <t>STRY2000001</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -4888,12 +4945,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>MISALIGNED</t>
+          <t>ALIGNED</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -4903,7 +4960,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Revised Edge Cases</t>
+          <t>Revised Core</t>
         </is>
       </c>
     </row>
@@ -4915,58 +4972,70 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>STRY2000004</t>
+          <t>STRY2000001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AU31</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+          <t>AU05</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>STRY2000001</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>NOT EXECUTED</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>NOT_EXECUTED</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>NOT_EXECUTED</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Revised Core</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>RLSE1000002</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>STRY2000005</t>
-        </is>
-      </c>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AU40</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>STRY2000005</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -4986,22 +5055,22 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>EXECUTION_ONLY</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Revised Edge Cases</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
     </row>
@@ -5013,27 +5082,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>STRY2000005</t>
+          <t>STRY2000002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AU41</t>
+          <t>AU10</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>STRY2000005</t>
+          <t>STRY2000002</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5070,41 +5139,750 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>STRY2000002</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>AU11</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>STRY2000002</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Revised Edge Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>STRY2000002</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>AU12</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>NEGATIVE</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>MISALIGNED</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Revised Edge Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TP-ORPHAN-01</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>STRY3999999</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>EXECUTION_ONLY</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>DS and Optimisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>STRY2000003</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>AU20</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>STRY2000003</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Revised Edge Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>STRY2000003</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AU21</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>STRY2000004</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>MISALIGNED</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Revised Edge Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TP-ORPHAN-01</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>STRY3999999</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>EXECUTION_ONLY</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>DS and Optimisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>STRY2000004</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>AU30</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>STRY2000004</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Revised Edge Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>STRY2000004</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AU30</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>STRY2000002</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>MISALIGNED</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Revised Edge Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>STRY2000004</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>AU31</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>NOT EXECUTED</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>NOT_EXECUTED</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>NOT_EXECUTED</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>TP-ORPHAN-01</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>STRY3999999</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>EXECUTION_ONLY</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>DS and Optimisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>STRY2000005</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>AU40</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>STRY2000005</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Revised Edge Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>STRY2000005</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AU41</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>STRY2000005</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Audit Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Revised Edge Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>RLSE1000002</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>STRY2000005</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
         <is>
           <t>AU42</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>NOT_EXECUTED</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr">
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>NOT_EXECUTED</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>TP-ORPHAN-01</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>STRY3999999</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>EXECUTION_ONLY</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>DS and Optimisation</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K37"/>
+  <autoFilter ref="A1:K50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5115,7 +5893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -5126,7 +5904,7 @@
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
@@ -5888,8 +6666,58 @@
         <v>1</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>UNREFERENCED</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>STRY3999999</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>DS and Optimisation</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>TP-ORPHAN-01</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>TP-ORPHAN-01</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N14"/>
+  <autoFilter ref="A1:N15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5946,10 +6774,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5980,8 +6808,15 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TP-ORPHAN-01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:A4"/>
+  <autoFilter ref="A1:A5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6607,13 +7442,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -7785,20 +8620,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Phase A</t>
+          <t>DS and Optimisation</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>STRY1000001</t>
+          <t>STRY3999999</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>EX01</t>
+          <t>TP-ORPHAN-01</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7808,17 +8643,17 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
+          <t>Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Evidenced</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -7829,7 +8664,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -7838,7 +8673,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>EX02</t>
+          <t>EX01</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7869,7 +8704,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -7878,7 +8713,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>EX03</t>
+          <t>EX02</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7905,20 +8740,20 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Phase B</t>
+          <t>Phase A</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>STRY1000002</t>
+          <t>STRY1000001</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>EX10</t>
+          <t>EX03</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7949,7 +8784,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -7958,7 +8793,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>EX11</t>
+          <t>EX10</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7989,7 +8824,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -7998,7 +8833,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>EX12</t>
+          <t>EX11</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -8029,16 +8864,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>STRY1000003</t>
+          <t>STRY1000002</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>EX20</t>
+          <t>EX12</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -8069,41 +8904,81 @@
         </is>
       </c>
       <c r="B37" t="n">
+        <v>5</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>STRY1000003</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>EX20</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Evidenced</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Phase B</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
         <v>6</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>STRY1000003</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>EX21</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
         <is>
           <t>Extraction Validation Test Assurance Scripts v0.3.xlsx</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>Evidenced</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H37"/>
+  <autoFilter ref="A1:H38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>